<commit_message>
Update AI Multi-Agent DSS project
</commit_message>
<xml_diff>
--- a/datasets/sales_data.xlsx
+++ b/datasets/sales_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8118dd153ecada9/Desktop/AI_MultiAgent_DSS/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7121192F-2449-429B-B6D4-F5DFE7E57B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7121192F-2449-429B-B6D4-F5DFE7E57B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBBDFC26-9B78-4805-A1B9-EC0DFA94C619}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="816" windowWidth="9156" windowHeight="8880" xr2:uid="{0B95B12E-178E-434C-998E-666771B81B44}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{0B95B12E-178E-434C-998E-666771B81B44}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>